<commit_message>
Use Woningborg 2027 tariffs in comparison: single rate per regeling over koop-/aanneemsom, high-rise rate, VAT and additional costs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D1yv8wu8NwMW66m8HY524p
</commit_message>
<xml_diff>
--- a/templates/Tariefvergelijking_SWK_Woningborg.xlsx
+++ b/templates/Tariefvergelijking_SWK_Woningborg.xlsx
@@ -14,14 +14,34 @@
     <sheet name="Toelichting" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Tarieven SWK'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Tarieven Woningborg'!$A$1:$I$36</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Vergelijking!$A$1:$H$54</definedName>
-    <definedName function="false" hidden="false" name="AanneemsomIncl" vbProcedure="false">Vergelijking!$D$15</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Tarieven SWK'!$A$1:$I$37</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Tarieven Woningborg'!$A$1:$I$45</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Vergelijking!$A$1:$H$56</definedName>
+    <definedName function="false" hidden="false" name="AanneemsomExcl" vbProcedure="false">Vergelijking!$D$13</definedName>
+    <definedName function="false" hidden="false" name="AanneemsomIncl" vbProcedure="false">Vergelijking!$D$16</definedName>
     <definedName function="false" hidden="false" name="AantalWoningen" vbProcedure="false">Vergelijking!$D$12</definedName>
+    <definedName function="false" hidden="false" name="Bouwlagen" vbProcedure="false">Vergelijking!$D$18</definedName>
+    <definedName function="false" hidden="false" name="BtwKoopsom" vbProcedure="false">Vergelijking!$C$15</definedName>
+    <definedName function="false" hidden="false" name="GrondExcl" vbProcedure="false">Vergelijking!$D$14</definedName>
     <definedName function="false" hidden="false" name="KeuzeBouwtijd" vbProcedure="false">Vergelijking!$H$13</definedName>
-    <definedName function="false" hidden="false" name="KeuzeHoogbouw" vbProcedure="false">Vergelijking!$H$11</definedName>
+    <definedName function="false" hidden="false" name="KeuzeHoogbouw" vbProcedure="false">Vergelijking!$H$14</definedName>
     <definedName function="false" hidden="false" name="KeuzeZakelijk" vbProcedure="false">Vergelijking!$H$12</definedName>
+    <definedName function="false" hidden="false" name="KoopAanneemIncl" vbProcedure="false">Vergelijking!$D$17</definedName>
+    <definedName function="false" hidden="false" name="SWK_Btw" vbProcedure="false">'Tarieven SWK'!$H$36</definedName>
+    <definedName function="false" hidden="false" name="SWK_Excl" vbProcedure="false">'Tarieven SWK'!$H$35</definedName>
+    <definedName function="false" hidden="false" name="SWK_Incl" vbProcedure="false">'Tarieven SWK'!$H$37</definedName>
+    <definedName function="false" hidden="false" name="SWK_Opslag" vbProcedure="false">'Tarieven SWK'!$H$23</definedName>
+    <definedName function="false" hidden="false" name="SWK_Overig" vbProcedure="false">'Tarieven SWK'!$H$33</definedName>
+    <definedName function="false" hidden="false" name="SWK_Premie" vbProcedure="false">('Tarieven SWK'!$G$12+'Tarieven SWK'!$G$13)</definedName>
+    <definedName function="false" hidden="false" name="WB_Btw" vbProcedure="false">'Tarieven Woningborg'!$H$44</definedName>
+    <definedName function="false" hidden="false" name="WB_Excl" vbProcedure="false">'Tarieven Woningborg'!$H$43</definedName>
+    <definedName function="false" hidden="false" name="WB_GrondslagSoort" vbProcedure="false">'Tarieven Woningborg'!$D$25</definedName>
+    <definedName function="false" hidden="false" name="WB_Hoog" vbProcedure="false">Vergelijking!$H$17</definedName>
+    <definedName function="false" hidden="false" name="WB_Incl" vbProcedure="false">'Tarieven Woningborg'!$H$45</definedName>
+    <definedName function="false" hidden="false" name="WB_Opslag" vbProcedure="false">0</definedName>
+    <definedName function="false" hidden="false" name="WB_Overig" vbProcedure="false">'Tarieven Woningborg'!$H$40</definedName>
+    <definedName function="false" hidden="false" name="WB_Premie" vbProcedure="false">'Tarieven Woningborg'!$H$27</definedName>
+    <definedName function="false" hidden="false" name="WB_Regeling" vbProcedure="false">Vergelijking!$H$16</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -33,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="170">
   <si>
     <t xml:space="preserve">HEIJMANS  |  VASTGOED</t>
   </si>
@@ -41,13 +61,13 @@
     <t xml:space="preserve">Vergelijking SWK  vs.  Woningborg  |  Garantie- en Waarborgregeling</t>
   </si>
   <si>
-    <t xml:space="preserve">Blauwe cijfers op geel = invoer  ·  Tarieven staan op de tabbladen 'Tarieven SWK' en 'Tarieven Woningborg'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAAL SWK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAAL WONINGBORG</t>
+    <t xml:space="preserve">Blauwe cijfers op geel = invoer  ·  Tarieven: 'Tarieven SWK' (rekenmodel 2026) en 'Tarieven Woningborg' (tarievenbrief 2027)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWK  (EXCL. BTW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WONINGBORG  (EXCL. BTW)</t>
   </si>
   <si>
     <t xml:space="preserve">VERSCHIL</t>
@@ -68,138 +88,198 @@
     <t xml:space="preserve">Voorbeeldproject</t>
   </si>
   <si>
-    <t xml:space="preserve">Hoogbouw (&gt; 13 bouwlagen)</t>
+    <t xml:space="preserve">SWK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aantal woningen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verlengde garantie zakelijk</t>
   </si>
   <si>
     <t xml:space="preserve">nee</t>
   </si>
   <si>
-    <t xml:space="preserve">Aantal woningen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zakelijke opdrachtgever (verlengde garantie)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Aanneemsom (excl. btw)</t>
   </si>
   <si>
     <t xml:space="preserve">Prognose bouwtijd &gt; 3 jaar</t>
   </si>
   <si>
+    <t xml:space="preserve">Koopsom grond (excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoogbouwopslag (&gt; 13 bouwlagen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Woningborg</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aanneemsom (incl. btw)</t>
   </si>
   <si>
+    <t xml:space="preserve">Regeling / certificaat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Particulier nieuwbouw – verkoop met grond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koop- en aanneemsom (incl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoogbouwtarief (vanaf 13 lagen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aantal bouwlagen boven straatpeil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grondslag premie</t>
+  </si>
+  <si>
     <t xml:space="preserve">KOSTENVERGELIJKING</t>
   </si>
   <si>
     <t xml:space="preserve">Kostenpost</t>
   </si>
   <si>
-    <t xml:space="preserve">SWK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Woningborg</t>
-  </si>
-  <si>
     <t xml:space="preserve">Verschil (WB − SWK)</t>
   </si>
   <si>
     <t xml:space="preserve">Voordeligst</t>
   </si>
   <si>
+    <t xml:space="preserve">Toelichting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provisie / premie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWK: Sectie I + II  ·  WB: tarief × grondslag regeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opslagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WB: hoogbouw zit in het tarief zelf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overige / bijkomende kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWK: bureaukosten  ·  WB: bezoeken, metingen, diensten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totaal excl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relevante vergelijking als de btw aftrekbaar is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Btw over tarieven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentages: zie de tariefbladen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totaal incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kosten per woning (excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In % van aanneemsom incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelfde noemer voor beide, zodat ze vergelijkbaar zijn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positief verschil = Woningborg duurder; negatief = Woningborg goedkoper.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONTROLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LET OP: VERSCHILLEN IN REKENWIJZE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoer compleet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• SWK: twee provisies + opslagen over de aanneemsom. WB: één tarief over de koop- én aanneemsom.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keuzes geldig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• WB rekent btw over de premie; het SWK-rekenmodel noemt geen btw (staat op 0%, controleren).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarieven SWK bevestigd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Hoogbouw: SWK-opslag bij &gt; 13 lagen, WB-hoogbouwtarief vanaf 13 lagen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarieven Woningborg bevestigd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Tariefjaar verschilt: SWK 2026 (rekenmodel), Woningborg 2027 (tarievenbrief).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koopsom grond ingevuld (bij 'met grond')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• WB-bouwplaatsbezoeken/geluidsmetingen alleen bij transformatie en houtbouw (op offerte).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarieven SWK  |  Garantie- en Waarborgregeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blauwe cijfers op geel = tarief/keuze aanpassen  ·  Lichtblauw = berekening (rekent met de invoer op 'Vergelijking')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bron / tarieflijst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWK Rekenmodel 2026 – Berekening Garantie- en Waarborgregeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bevestigd?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Het SWK-rekenmodel noemt geen btw over de provisie; controleren en zo nodig op 21% zetten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BASISPROVISIES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grondslag %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grondslag (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bedrag (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(grondslag = % van de aanneemsom incl. btw)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Provisie Sectie I (Afbouw)</t>
   </si>
   <si>
+    <t xml:space="preserve">Over 20% van de aanneemsom incl. btw</t>
+  </si>
+  <si>
     <t xml:space="preserve">Provisie Sectie II (Kwaliteit)</t>
   </si>
   <si>
-    <t xml:space="preserve">Opslagen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overige kosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totaal kosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kosten per woning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In % van aanneemsom incl. btw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Positief verschil = Woningborg duurder; negatief = Woningborg goedkoper. Bedragen zoals de tarieflijsten, excl. eventuele btw.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONTROLES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AANDACHTSPUNTEN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invoer compleet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Woningborg-tarieven zijn voorbeeldwaarden tot ze zijn bevestigd.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keuzes geldig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Technische beoordeling (transformatie, &gt; 25 lagen) niet inbegrepen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarieven SWK bevestigd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Alleen volledige regeling; geen separaat verkochte parkeerplaatsen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarieven Woningborg bevestigd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarieven SWK  |  Garantie- en Waarborgregeling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blauwe cijfers op geel = tarief/keuze aanpassen  ·  Lichtblauw = berekening (rekent met de invoer op 'Vergelijking')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bron / tarieflijst</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SWK Rekenmodel 2026 – Berekening Garantie- en Waarborgregeling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bevestigd?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BASISPROVISIES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grondslag %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grondslag (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bedrag (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toelichting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(grondslag = % van de aanneemsom incl. btw)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Over 20% van de aanneemsom incl. btw</t>
-  </si>
-  <si>
     <t xml:space="preserve">Over de aanneemsom incl. btw</t>
   </si>
   <si>
@@ -227,7 +307,7 @@
     <t xml:space="preserve">Hoogbouw</t>
   </si>
   <si>
-    <t xml:space="preserve">&gt; 13 bouwlagen</t>
+    <t xml:space="preserve">&gt; 13 bouwlagen (volgt uit aantal bouwlagen)</t>
   </si>
   <si>
     <t xml:space="preserve">Opslag verlengde garantie zakelijk</t>
@@ -278,37 +358,166 @@
     <t xml:space="preserve">Voorschot per woning</t>
   </si>
   <si>
-    <t xml:space="preserve">Totaal kosten SWK</t>
+    <t xml:space="preserve">Totaal kosten SWK (excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totaal kosten SWK (incl. btw)</t>
   </si>
   <si>
     <t xml:space="preserve">Tarieven Woningborg  |  Garantie- en Waarborgregeling</t>
   </si>
   <si>
-    <t xml:space="preserve">VOORBEELD – vul hier de actuele Woningborg-tarieflijst in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠  VOORBEELDTARIEVEN – dit zijn géén officiële Woningborg-tarieven. Vervang ze en zet 'Bevestigd' op ja.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provisie insolventiedeel / afbouw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VOORBEELDWAARDE – controleren</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provisie herstel-/kwaliteitsdeel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opslag zakelijke opdrachtgever</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opslag lange bouwtijd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registratie-/bureaukosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totaal kosten Woningborg</t>
+    <t xml:space="preserve">Tarievenbrief Woningborg Verzekeren 2027 (18-09-2026), Heijmans Vastgoed – inschrijfnr. 4889</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volgens de tarievenbrief: 'Over alle tarieven wordt btw in rekening gebracht'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geldig voor plannen geaccepteerd op of na 1 januari 2027. Particulier: grondslag incl. meer-/minderwerk en btw. Zakelijk: grondslag excl. btw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARIEFMATRIX 2027  (% van de grondslag)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tot 13 lagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vanaf 13 lagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grondslag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(kies de regeling op het tabblad 'Vergelijking')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koop- en aanneemsom incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ook bij afgekochte erfpachtcanon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Particulier nieuwbouw – verkoop zonder grond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aanneemsom incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grond door derde verkocht / erfpacht zonder afkoop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kavelbouw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transformatie particulier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ook zonder grond over koop- en aanneemsom; + bijkomende kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zakelijk nieuwbouw – insolventie + herstel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aanneemsom excl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zakelijk nieuwbouw – alleen insolventie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zakelijk transformatie – insolventie + herstel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koop- en aanneemsom excl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gebouw valt WEL onder dekking; + bijkomende kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zakelijk transformatie – alleen insolventie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gebouw valt NIET onder dekking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREMIEBEREKENING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gekozen regeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soort grondslag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIJKOMENDE KOSTEN EN EXTRA DIENSTVERLENING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wanneer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totaal (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bouwplaatsbezoek (per bezoek)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transformatie / houtbouw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Op offerte na eerste opname</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geluidsmeting (per meting)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transformatie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opstellen depotovereenkomst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Op verzoek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eenmalig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opstellen afbouwverklaring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laten vervallen van plan na risicobeoordeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planacceptatie bij &lt; 70% verkocht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aanpassing standaard termijnregeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaarlijkse bijdrage (per onderneming)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per jaar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niet projectgebonden; standaard niet meegeteld</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inschrijfgeld (per onderneming)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binnen concern € 1.133 per extra inschrijving</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alle bedragen excl. btw. Vul bij 'Aantal' in wat voor dit project verwacht wordt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totaal kosten Woningborg (excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totaal kosten Woningborg (incl. btw)</t>
   </si>
   <si>
     <t xml:space="preserve">Hoe werkt deze vergelijking?</t>
@@ -317,47 +526,50 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">Vul op 'Vergelijking' het project in: aantal woningen, aanneemsom excl. btw, btw-% en de drie keuzes (ja/nee).</t>
+    <t xml:space="preserve">Vul op 'Vergelijking' het project in: aantal woningen, aanneemsom en koopsom grond (excl. btw), btw-% en aantal bouwlagen.</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">Controleer op 'Tarieven SWK' en 'Tarieven Woningborg' de percentages en bedragen; zet 'Bevestigd' op ja als ze kloppen.</t>
+    <t xml:space="preserve">Kies de SWK-keuzes (zakelijk, bouwtijd) en de Woningborg-regeling. Hoogbouw volgt automatisch uit het aantal bouwlagen.</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
-    <t xml:space="preserve">Opslagen: kies waarover ze worden berekend (Sectie I, Sectie II of aanneemsom) en wanneer ze gelden (Altijd, of gekoppeld aan een keuze).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overige kosten: bedrag per woning of per project, eventueel gekoppeld aan een keuze.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">i</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SWK-tarieven zijn overgenomen uit het rekenmodel 2026 (Sectie I 0,5198% over 20%, Sectie II 0,0380%, opslagen 30,3% / 10% / 10%, bureaukosten € 750).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Woningborg-tarieven zijn VOORBEELDWAARDEN in dezelfde opbouw, geen officiële tarieven. De controle op 'Vergelijking' blijft rood tot ze bevestigd zijn.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sectie I/II zijn SWK-termen; gebruik bij Woningborg de twee basisregels voor hun equivalent (insolventie-/afbouwdeel en herstel-/kwaliteitsdeel).</t>
+    <t xml:space="preserve">Vul op 'Tarieven Woningborg' bij 'Aantal' de verwachte bijkomende kosten in (bezoeken, metingen, extra diensten).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verschil in rekenwijze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWK: provisie Sectie I (0,5198% over 20% van de aanneemsom) + Sectie II (0,0380% over de aanneemsom) + opslagen + € 750 bureaukosten per woning.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Woningborg: één tarief per regeling over de koop- en aanneemsom (met grond) of de aanneemsom (zonder grond / kavelbouw). Hoogbouw (≥ 13 lagen) = hoger tarief, geen opslag.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Woningborg particulier rekent over de som incl. btw en meer-/minderwerk, zakelijk over de som excl. btw. Over de premie zelf komt btw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De SWK-provisie staat zonder btw (0%), zoals in het SWK-rekenmodel. Controleer of SWK btw rekent en pas het percentage op 'Tarieven SWK' zo nodig aan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tariefjaren: SWK 2026 (rekenmodel), Woningborg 2027 (tarievenbrief 18-09-2026). Werk de SWK-tarieven bij zodra die voor 2027 bekend zijn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niet meegenomen: houtbouwtoeslag van Woningborg (na technische beoordeling) en SWK-beoordelingen (transformatie, hoogbouw &gt; 25 lagen, afwijkende termijnregeling).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;€ &quot;#,##0;[RED]&quot;(€ &quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
@@ -366,8 +578,9 @@
     <numFmt numFmtId="169" formatCode="&quot;€ &quot;#,##0"/>
     <numFmt numFmtId="170" formatCode="0.0000%"/>
     <numFmt numFmtId="171" formatCode="0.0%"/>
+    <numFmt numFmtId="172" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -469,8 +682,33 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF003B5C"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF4A4F55"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FFC98A00"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -514,6 +752,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF4A4F55"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF111F39"/>
@@ -529,8 +774,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF4A4F55"/>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -549,22 +794,8 @@
       <family val="2"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <i val="true"/>
       <sz val="8"/>
-      <color rgb="FF4A4F55"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FF4A4F55"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -577,8 +808,15 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF111F39"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -618,13 +856,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF3C4"/>
-        <bgColor rgb="FFFFFF99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC0392B"/>
-        <bgColor rgb="FF993366"/>
+        <bgColor rgb="FFFDE9B8"/>
       </patternFill>
     </fill>
   </fills>
@@ -709,7 +941,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="71">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -774,71 +1006,87 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="16" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="24" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -846,27 +1094,35 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -874,67 +1130,99 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -947,7 +1235,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
     <dxf>
       <font>
         <b val="1"/>
@@ -1001,6 +1289,16 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFDE9B8"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <colors>
     <indexedColors>
@@ -1039,7 +1337,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFD9EAD3"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFDE9B8"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -1056,7 +1354,7 @@
       <rgbColor rgb="FF38761D"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FFC0392B"/>
+      <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF111F39"/>
@@ -1115,7 +1413,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Vergelijking!C19</c:f>
+              <c:f>Vergelijking!C21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1162,40 +1460,34 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Vergelijking!$B$20:$B$23</c:f>
+              <c:f>Vergelijking!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Provisie Sectie I (Afbouw)</c:v>
+                  <c:v>Provisie / premie</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Provisie Sectie II (Kwaliteit)</c:v>
+                  <c:v>Opslagen</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Opslagen</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Overige kosten</c:v>
+                  <c:v>Overige / bijkomende kosten</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Vergelijking!$C$20:$C$23</c:f>
+              <c:f>Vergelijking!$C$22:$C$24</c:f>
               <c:numCache>
                 <c:formatCode>"€ "#,##0;[RED]"(€ "#,##0\);\-</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>528.32472</c:v>
+                  <c:v>721.44072</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>193.116</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>750</c:v>
                 </c:pt>
               </c:numCache>
@@ -1207,7 +1499,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Vergelijking!D19</c:f>
+              <c:f>Vergelijking!D21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1254,41 +1546,35 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Vergelijking!$B$20:$B$23</c:f>
+              <c:f>Vergelijking!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Provisie Sectie I (Afbouw)</c:v>
+                  <c:v>Provisie / premie</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Provisie Sectie II (Kwaliteit)</c:v>
+                  <c:v>Opslagen</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Opslagen</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Overige kosten</c:v>
+                  <c:v>Overige / bijkomende kosten</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Vergelijking!$D$20:$D$23</c:f>
+              <c:f>Vergelijking!$D$22:$D$24</c:f>
               <c:numCache>
                 <c:formatCode>"€ "#,##0;[RED]"(€ "#,##0\);\-</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>508.2</c:v>
+                  <c:v>1373.35</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>203.28</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>700</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1296,11 +1582,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="84445910"/>
-        <c:axId val="47069330"/>
+        <c:axId val="89272089"/>
+        <c:axId val="59208267"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="84445910"/>
+        <c:axId val="89272089"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1332,7 +1618,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47069330"/>
+        <c:crossAx val="59208267"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1340,7 +1626,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47069330"/>
+        <c:axId val="59208267"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1372,7 +1658,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84445910"/>
+        <c:crossAx val="89272089"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1430,14 +1716,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>2014200</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>42840</xdr:rowOff>
+      <xdr:colOff>1943640</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>43200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1445,7 +1731,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="141120" y="9296280"/>
+        <a:off x="141120" y="9725040"/>
         <a:ext cx="8639640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1640,16 +1926,16 @@
     <tabColor rgb="FFFEB900"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:H37"/>
+  <dimension ref="B1:H38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1713,21 +1999,21 @@
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="n">
-        <f aca="false">C25</f>
+        <f aca="false">SWK_Excl</f>
         <v>1471.44072</v>
       </c>
       <c r="C6" s="9" t="n">
-        <f aca="false">D25</f>
-        <v>1411.48</v>
+        <f aca="false">WB_Excl</f>
+        <v>1373.35</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="10" t="n">
-        <f aca="false">ABS(E25)</f>
-        <v>59.96072</v>
+        <f aca="false">ABS(WB_Excl-SWK_Excl)</f>
+        <v>98.0907200000002</v>
       </c>
       <c r="F6" s="10"/>
       <c r="G6" s="11" t="str">
-        <f aca="false">IF(C25=D25,"Gelijk",IF(C25&lt;D25,"SWK","Woningborg"))</f>
+        <f aca="false">IF(SWK_Excl=WB_Excl,"Gelijk",IF(SWK_Excl&lt;WB_Excl,"SWK","Woningborg"))</f>
         <v>Woningborg</v>
       </c>
       <c r="H6" s="11"/>
@@ -1746,8 +2032,8 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="12" t="str">
-        <f aca="false">IF(MAX(C25:D25)=0,"",TEXT(ABS(E25)/MAX(C25:D25),"0.0%")&amp;" goedkoper")</f>
-        <v>4.1% goedkoper</v>
+        <f aca="false">IF(MAX(SWK_Excl,WB_Excl)=0,"",TEXT(ABS(WB_Excl-SWK_Excl)/MAX(SWK_Excl,WB_Excl),"0.0%")&amp;" goedkoper")</f>
+        <v>6.7% goedkoper</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -1785,16 +2071,14 @@
       <c r="D11" s="15"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H11" s="16" t="s">
-        <v>12</v>
-      </c>
+      <c r="H11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="17" t="n">
@@ -1803,10 +2087,10 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="18" t="s">
         <v>14</v>
-      </c>
-      <c r="H12" s="16" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1814,7 +2098,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="19" t="n">
         <v>420000</v>
       </c>
       <c r="E13" s="4"/>
@@ -1822,284 +2106,343 @@
       <c r="G13" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="16" t="s">
-        <v>12</v>
+      <c r="H13" s="18" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="14" t="str">
-        <f aca="false">"Btw ("&amp;TEXT(C14,"0%")&amp;")"</f>
-        <v>Btw (21%)</v>
-      </c>
-      <c r="C14" s="19" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="D14" s="20" t="n">
-        <f aca="false">D13*C14</f>
-        <v>88200</v>
+      <c r="B14" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="19" t="n">
+        <v>80000</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+      <c r="G14" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="20" t="str">
+        <f aca="false">IF(Bouwlagen&gt;13,"ja","nee")</f>
+        <v>nee</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="4"/>
+      <c r="B15" s="14" t="str">
+        <f aca="false">"Btw op koop-/aanneemsom ("&amp;TEXT(C15,"0%")&amp;")"</f>
+        <v>Btw op koop-/aanneemsom (21%)</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>0.21</v>
+      </c>
       <c r="D15" s="22" t="n">
-        <f aca="false">D13+D14</f>
-        <v>508200</v>
+        <f aca="false">(D13+D14)*C15</f>
+        <v>105000</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
+      <c r="G15" s="23" t="s">
+        <v>19</v>
+      </c>
       <c r="H15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4"/>
+      <c r="B16" s="24" t="s">
+        <v>20</v>
+      </c>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="25" t="n">
+        <f aca="false">D13*(1+C15)</f>
+        <v>508200</v>
+      </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
+      <c r="G16" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="4"/>
+      <c r="B17" s="24" t="s">
+        <v>23</v>
+      </c>
       <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+      <c r="D17" s="25" t="n">
+        <f aca="false">(D13+D14)*(1+C15)</f>
+        <v>605000</v>
+      </c>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
+      <c r="G17" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="H17" s="20" t="str">
+        <f aca="false">IF(Bouwlagen&gt;=13,"ja","nee")</f>
+        <v>nee</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="H18" s="20" t="str">
+        <f aca="false">WB_GrondslagSoort</f>
+        <v>Koop- en aanneemsom incl. btw</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+    </row>
+    <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="E19" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" s="27"/>
-    </row>
-    <row r="20" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="28" t="n">
-        <f aca="false">'Tarieven SWK'!G12</f>
-        <v>528.32472</v>
-      </c>
-      <c r="D20" s="28" t="n">
-        <f aca="false">'Tarieven Woningborg'!G12</f>
-        <v>508.2</v>
-      </c>
-      <c r="E20" s="29" t="n">
-        <f aca="false">D20-C20</f>
-        <v>-20.1247200000001</v>
-      </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="30" t="str">
-        <f aca="false">IF(C20=D20,"–",IF(C20&lt;D20,"SWK","Woningborg"))</f>
-        <v>Woningborg</v>
-      </c>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="28" t="n">
-        <f aca="false">'Tarieven SWK'!G13</f>
-        <v>193.116</v>
-      </c>
-      <c r="D21" s="28" t="n">
-        <f aca="false">'Tarieven Woningborg'!G13</f>
-        <v>203.28</v>
-      </c>
-      <c r="E21" s="29" t="n">
-        <f aca="false">D21-C21</f>
-        <v>10.164</v>
-      </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="30" t="str">
-        <f aca="false">IF(C21=D21,"–",IF(C21&lt;D21,"SWK","Woningborg"))</f>
-        <v>SWK</v>
-      </c>
-      <c r="H21" s="4"/>
+      <c r="E21" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" s="29"/>
+      <c r="G21" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="H21" s="26" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="28" t="n">
-        <f aca="false">'Tarieven SWK'!H23</f>
-        <v>0</v>
-      </c>
-      <c r="D22" s="28" t="n">
-        <f aca="false">'Tarieven Woningborg'!H23</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="C22" s="31" t="n">
+        <f aca="false">SWK_Premie</f>
+        <v>721.44072</v>
+      </c>
+      <c r="D22" s="31" t="n">
+        <f aca="false">WB_Premie</f>
+        <v>1373.35</v>
+      </c>
+      <c r="E22" s="32" t="n">
         <f aca="false">D22-C22</f>
-        <v>0</v>
+        <v>651.90928</v>
       </c>
       <c r="F22" s="4"/>
-      <c r="G22" s="30" t="str">
+      <c r="G22" s="33" t="str">
         <f aca="false">IF(C22=D22,"–",IF(C22&lt;D22,"SWK","Woningborg"))</f>
-        <v>–</v>
-      </c>
-      <c r="H22" s="4"/>
+        <v>SWK</v>
+      </c>
+      <c r="H22" s="34" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23" s="28" t="n">
-        <f aca="false">'Tarieven SWK'!H33</f>
+        <v>34</v>
+      </c>
+      <c r="C23" s="31" t="n">
+        <f aca="false">SWK_Opslag</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="31" t="n">
+        <f aca="false">WB_Opslag</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="32" t="n">
+        <f aca="false">D23-C23</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="4"/>
+      <c r="G23" s="33" t="str">
+        <f aca="false">IF(C23=D23,"–",IF(C23&lt;D23,"SWK","Woningborg"))</f>
+        <v>–</v>
+      </c>
+      <c r="H23" s="34" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" s="31" t="n">
+        <f aca="false">SWK_Overig</f>
         <v>750</v>
       </c>
-      <c r="D23" s="28" t="n">
-        <f aca="false">'Tarieven Woningborg'!H33</f>
-        <v>700</v>
-      </c>
-      <c r="E23" s="29" t="n">
-        <f aca="false">D23-C23</f>
-        <v>-50</v>
-      </c>
-      <c r="F23" s="4"/>
-      <c r="G23" s="30" t="str">
-        <f aca="false">IF(C23=D23,"–",IF(C23&lt;D23,"SWK","Woningborg"))</f>
+      <c r="D24" s="31" t="n">
+        <f aca="false">WB_Overig</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="32" t="n">
+        <f aca="false">D24-C24</f>
+        <v>-750</v>
+      </c>
+      <c r="F24" s="4"/>
+      <c r="G24" s="33" t="str">
+        <f aca="false">IF(C24=D24,"–",IF(C24&lt;D24,"SWK","Woningborg"))</f>
         <v>Woningborg</v>
       </c>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-    </row>
-    <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="32" t="n">
-        <f aca="false">SUM(C20:C23)</f>
+      <c r="H24" s="34" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="36" t="n">
+        <f aca="false">SUM(C22:C24)</f>
         <v>1471.44072</v>
       </c>
-      <c r="D25" s="32" t="n">
-        <f aca="false">SUM(D20:D23)</f>
-        <v>1411.48</v>
-      </c>
-      <c r="E25" s="32" t="n">
-        <f aca="false">D25-C25</f>
-        <v>-59.96072</v>
-      </c>
-      <c r="F25" s="33"/>
-      <c r="G25" s="34" t="str">
-        <f aca="false">IF(C25=D25,"–",IF(C25&lt;D25,"SWK","Woningborg"))</f>
+      <c r="D26" s="36" t="n">
+        <f aca="false">SUM(D22:D24)</f>
+        <v>1373.35</v>
+      </c>
+      <c r="E26" s="36" t="n">
+        <f aca="false">D26-C26</f>
+        <v>-98.0907200000002</v>
+      </c>
+      <c r="F26" s="37"/>
+      <c r="G26" s="38" t="str">
+        <f aca="false">IF(C26=D26,"–",IF(C26&lt;D26,"SWK","Woningborg"))</f>
         <v>Woningborg</v>
       </c>
-      <c r="H25" s="33"/>
-    </row>
-    <row r="26" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="20" t="n">
-        <f aca="false">IFERROR(C25/AantalWoningen,0)</f>
-        <v>1471.44072</v>
-      </c>
-      <c r="D26" s="20" t="n">
-        <f aca="false">IFERROR(D25/AantalWoningen,0)</f>
-        <v>1411.48</v>
-      </c>
-      <c r="E26" s="29" t="n">
-        <f aca="false">D26-C26</f>
-        <v>-59.96072</v>
-      </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
+      <c r="H26" s="39" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="36" t="n">
-        <f aca="false">IFERROR(C25/AanneemsomIncl,0)</f>
-        <v>0.00289539693034239</v>
-      </c>
-      <c r="D27" s="36" t="n">
-        <f aca="false">IFERROR(D25/AanneemsomIncl,0)</f>
-        <v>0.00277741046831956</v>
-      </c>
-      <c r="E27" s="37" t="n">
+      <c r="B27" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="22" t="n">
+        <f aca="false">SWK_Btw</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <f aca="false">WB_Btw</f>
+        <v>288.4035</v>
+      </c>
+      <c r="E27" s="32" t="n">
         <f aca="false">D27-C27</f>
-        <v>-0.000117986462022825</v>
+        <v>288.4035</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
+      <c r="H27" s="34" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
+      <c r="B28" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="25" t="n">
+        <f aca="false">SWK_Incl</f>
+        <v>1471.44072</v>
+      </c>
+      <c r="D28" s="25" t="n">
+        <f aca="false">WB_Incl</f>
+        <v>1661.7535</v>
+      </c>
+      <c r="E28" s="41" t="n">
+        <f aca="false">D28-C28</f>
+        <v>190.31278</v>
+      </c>
       <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
+      <c r="G28" s="42" t="str">
+        <f aca="false">IF(C28=D28,"–",IF(C28&lt;D28,"SWK","Woningborg"))</f>
+        <v>SWK</v>
+      </c>
+      <c r="H28" s="34"/>
     </row>
     <row r="29" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
+      <c r="B29" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="22" t="n">
+        <f aca="false">IFERROR(C26/AantalWoningen,0)</f>
+        <v>1471.44072</v>
+      </c>
+      <c r="D29" s="22" t="n">
+        <f aca="false">IFERROR(D26/AantalWoningen,0)</f>
+        <v>1373.35</v>
+      </c>
+      <c r="E29" s="32" t="n">
+        <f aca="false">D29-C29</f>
+        <v>-98.0907200000002</v>
+      </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
+      <c r="H29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
+      <c r="B30" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="43" t="n">
+        <f aca="false">IFERROR(C26/AanneemsomIncl,0)</f>
+        <v>0.00289539693034239</v>
+      </c>
+      <c r="D30" s="43" t="n">
+        <f aca="false">IFERROR(D26/AanneemsomIncl,0)</f>
+        <v>0.00270238095238095</v>
+      </c>
+      <c r="E30" s="44" t="n">
+        <f aca="false">D30-C30</f>
+        <v>-0.000193015977961433</v>
+      </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
+      <c r="H30" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="4"/>
+      <c r="B31" s="34" t="s">
+        <v>46</v>
+      </c>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
@@ -2107,92 +2450,110 @@
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
     </row>
-    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
+    <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
-      <c r="G32" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="H32" s="13"/>
-    </row>
-    <row r="33" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" s="40"/>
-      <c r="D33" s="41" t="str">
-        <f aca="false">IF(AND(D13&gt;0,D12&gt;0),"OK","AANVULLEN")</f>
-        <v>OK</v>
-      </c>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="42" t="s">
-        <v>35</v>
-      </c>
-      <c r="H33" s="42"/>
+      <c r="G33" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="H33" s="13"/>
     </row>
     <row r="34" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="C34" s="40"/>
-      <c r="D34" s="41" t="str">
-        <f aca="false">IF(AND(OR(H11="ja",H11="nee"),OR(H12="ja",H12="nee"),OR(H13="ja",H13="nee")),"OK","CONTROLEREN")</f>
+      <c r="B34" s="45" t="s">
+        <v>49</v>
+      </c>
+      <c r="C34" s="46"/>
+      <c r="D34" s="47" t="str">
+        <f aca="false">IF(AND(D13&gt;0,D12&gt;0,D18&gt;0),"OK","AANVULLEN")</f>
         <v>OK</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
-      <c r="G34" s="42" t="s">
-        <v>37</v>
-      </c>
-      <c r="H34" s="42"/>
+      <c r="G34" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="H34" s="48"/>
     </row>
     <row r="35" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="39" t="s">
-        <v>38</v>
-      </c>
-      <c r="C35" s="40"/>
-      <c r="D35" s="41" t="str">
+      <c r="B35" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="C35" s="46"/>
+      <c r="D35" s="47" t="str">
+        <f aca="false">IF(AND(OR(H12="ja",H12="nee"),OR(H13="ja",H13="nee"),ISNUMBER(MATCH(H16,'Tarieven Woningborg'!$B$12:$B$19,0))),"OK","CONTROLEREN")</f>
+        <v>OK</v>
+      </c>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="H35" s="48"/>
+    </row>
+    <row r="36" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="45" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" s="46"/>
+      <c r="D36" s="47" t="str">
         <f aca="false">'Tarieven SWK'!H5</f>
         <v>OK</v>
       </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="42" t="s">
-        <v>39</v>
-      </c>
-      <c r="H35" s="42"/>
-    </row>
-    <row r="36" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="C36" s="40"/>
-      <c r="D36" s="41" t="str">
-        <f aca="false">'Tarieven Woningborg'!H5</f>
-        <v>CONTROLEREN</v>
-      </c>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
+      <c r="G36" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="H36" s="48"/>
     </row>
     <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
+      <c r="B37" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" s="46"/>
+      <c r="D37" s="47" t="str">
+        <f aca="false">'Tarieven Woningborg'!H5</f>
+        <v>OK</v>
+      </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
+      <c r="G37" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="H37" s="48"/>
+    </row>
+    <row r="38" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" s="46"/>
+      <c r="D38" s="47" t="str">
+        <f aca="false">IF(AND(WB_GrondslagSoort="Koop- en aanneemsom incl. btw",D14&lt;=0),"CONTROLEREN","OK")</f>
+        <v>OK</v>
+      </c>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="48" t="s">
+        <v>58</v>
+      </c>
+      <c r="H38" s="48"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
@@ -2206,12 +2567,14 @@
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="C11:D11"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B33:D33"/>
     <mergeCell ref="G33:H33"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="G35:H35"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G38:H38"/>
   </mergeCells>
   <conditionalFormatting sqref="G6">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -2221,30 +2584,34 @@
       <formula>G6="Woningborg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G20:G25">
+  <conditionalFormatting sqref="G22:G28">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>G20="SWK"</formula>
+      <formula>G22="SWK"</formula>
     </cfRule>
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>G20="Woningborg"</formula>
+      <formula>G22="Woningborg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E20:E27">
+  <conditionalFormatting sqref="E22:E30">
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>E20&lt;0</formula>
+      <formula>E22&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D33:D36">
+  <conditionalFormatting sqref="D34:D38">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
-      <formula>D33="OK"</formula>
+      <formula>D34="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
-      <formula>D33&lt;&gt;"OK"</formula>
+      <formula>D34&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H11:H13" type="list">
+  <dataValidations count="2">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H12:H13" type="list">
       <formula1>"ja,nee"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H16" type="list">
+      <formula1>'Tarieven Woningborg'!$B$12:$B$19</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2265,7 +2632,7 @@
     <tabColor rgb="FF003B5C"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:I36"/>
+  <dimension ref="B1:I37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2292,7 +2659,7 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2304,7 +2671,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -2326,29 +2693,35 @@
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
-      <c r="G5" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="44" t="str">
+      <c r="G5" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="50" t="str">
         <f aca="false">IF(I5="ja","OK","CONTROLEREN")</f>
         <v>OK</v>
       </c>
-      <c r="I5" s="16" t="s">
-        <v>46</v>
+      <c r="I5" s="18" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="B6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>65</v>
+      </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -2377,7 +2750,7 @@
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="13" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
@@ -2388,30 +2761,30 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="G10" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="H10" s="26"/>
-      <c r="I10" s="23" t="s">
-        <v>52</v>
+      <c r="B10" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="29"/>
+      <c r="I10" s="26" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="45" t="s">
-        <v>53</v>
+      <c r="B11" s="51" t="s">
+        <v>71</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -2423,50 +2796,50 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="46" t="n">
+        <v>72</v>
+      </c>
+      <c r="C12" s="52" t="n">
         <v>0.005198</v>
       </c>
-      <c r="D12" s="47" t="n">
+      <c r="D12" s="53" t="n">
         <v>0.2</v>
       </c>
       <c r="E12" s="4"/>
-      <c r="F12" s="48" t="n">
+      <c r="F12" s="54" t="n">
         <f aca="false">AanneemsomIncl*D12</f>
         <v>101640</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="22" t="n">
         <f aca="false">F12*C12</f>
         <v>528.32472</v>
       </c>
       <c r="H12" s="4"/>
-      <c r="I12" s="38" t="s">
-        <v>54</v>
+      <c r="I12" s="34" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="46" t="n">
+        <v>74</v>
+      </c>
+      <c r="C13" s="52" t="n">
         <v>0.00038</v>
       </c>
-      <c r="D13" s="47" t="n">
+      <c r="D13" s="53" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="4"/>
-      <c r="F13" s="48" t="n">
+      <c r="F13" s="54" t="n">
         <f aca="false">AanneemsomIncl*D13</f>
         <v>508200</v>
       </c>
-      <c r="G13" s="20" t="n">
+      <c r="G13" s="22" t="n">
         <f aca="false">F13*C13</f>
         <v>193.116</v>
       </c>
       <c r="H13" s="4"/>
-      <c r="I13" s="38" t="s">
-        <v>55</v>
+      <c r="I13" s="34" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2481,7 +2854,7 @@
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="13" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
@@ -2492,174 +2865,174 @@
       <c r="I15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C16" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="G16" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="H16" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>52</v>
+      <c r="B16" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="G16" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="I16" s="26" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="49" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="50" t="n">
+      <c r="B17" s="55" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" s="56" t="n">
         <v>0.303</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="F17" s="48" t="n">
+        <v>83</v>
+      </c>
+      <c r="F17" s="54" t="n">
         <f aca="false">IF(D17="Sectie I",$G$12,IF(D17="Sectie II",$G$13,IF(D17="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
         <v>193.116</v>
       </c>
-      <c r="G17" s="51" t="str">
+      <c r="G17" s="57" t="str">
         <f aca="false">IF(B17="","",IF(IF(E17="Altijd",1,IF(E17="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E17="Zakelijk",--(KeuzeZakelijk="ja"),IF(E17="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v>nee</v>
       </c>
-      <c r="H17" s="20" t="n">
+      <c r="H17" s="22" t="n">
         <f aca="false">IF(G17="ja",F17*C17,0)</f>
         <v>0</v>
       </c>
-      <c r="I17" s="38" t="s">
-        <v>64</v>
+      <c r="I17" s="34" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="49" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" s="50" t="n">
+      <c r="B18" s="55" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="56" t="n">
         <v>0.1</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="48" t="n">
+        <v>86</v>
+      </c>
+      <c r="F18" s="54" t="n">
         <f aca="false">IF(D18="Sectie I",$G$12,IF(D18="Sectie II",$G$13,IF(D18="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
         <v>193.116</v>
       </c>
-      <c r="G18" s="51" t="str">
+      <c r="G18" s="57" t="str">
         <f aca="false">IF(B18="","",IF(IF(E18="Altijd",1,IF(E18="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E18="Zakelijk",--(KeuzeZakelijk="ja"),IF(E18="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v>nee</v>
       </c>
-      <c r="H18" s="20" t="n">
+      <c r="H18" s="22" t="n">
         <f aca="false">IF(G18="ja",F18*C18,0)</f>
         <v>0</v>
       </c>
-      <c r="I18" s="38" t="s">
-        <v>67</v>
+      <c r="I18" s="34" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="49" t="s">
-        <v>68</v>
-      </c>
-      <c r="C19" s="50" t="n">
+      <c r="B19" s="55" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="56" t="n">
         <v>0.1</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="F19" s="48" t="n">
+        <v>90</v>
+      </c>
+      <c r="F19" s="54" t="n">
         <f aca="false">IF(D19="Sectie I",$G$12,IF(D19="Sectie II",$G$13,IF(D19="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
         <v>528.32472</v>
       </c>
-      <c r="G19" s="51" t="str">
+      <c r="G19" s="57" t="str">
         <f aca="false">IF(B19="","",IF(IF(E19="Altijd",1,IF(E19="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E19="Zakelijk",--(KeuzeZakelijk="ja"),IF(E19="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v>nee</v>
       </c>
-      <c r="H19" s="20" t="n">
+      <c r="H19" s="22" t="n">
         <f aca="false">IF(G19="ja",F19*C19,0)</f>
         <v>0</v>
       </c>
-      <c r="I19" s="38" t="s">
-        <v>71</v>
+      <c r="I19" s="34" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="49"/>
-      <c r="C20" s="50"/>
+      <c r="B20" s="55"/>
+      <c r="C20" s="56"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
-      <c r="F20" s="48" t="n">
+      <c r="F20" s="54" t="n">
         <f aca="false">IF(D20="Sectie I",$G$12,IF(D20="Sectie II",$G$13,IF(D20="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
         <v>0</v>
       </c>
-      <c r="G20" s="51" t="str">
+      <c r="G20" s="57" t="str">
         <f aca="false">IF(B20="","",IF(IF(E20="Altijd",1,IF(E20="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E20="Zakelijk",--(KeuzeZakelijk="ja"),IF(E20="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H20" s="20" t="n">
+      <c r="H20" s="22" t="n">
         <f aca="false">IF(G20="ja",F20*C20,0)</f>
         <v>0</v>
       </c>
-      <c r="I20" s="38"/>
+      <c r="I20" s="34"/>
     </row>
     <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="49"/>
-      <c r="C21" s="50"/>
+      <c r="B21" s="55"/>
+      <c r="C21" s="56"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
-      <c r="F21" s="48" t="n">
+      <c r="F21" s="54" t="n">
         <f aca="false">IF(D21="Sectie I",$G$12,IF(D21="Sectie II",$G$13,IF(D21="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
         <v>0</v>
       </c>
-      <c r="G21" s="51" t="str">
+      <c r="G21" s="57" t="str">
         <f aca="false">IF(B21="","",IF(IF(E21="Altijd",1,IF(E21="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E21="Zakelijk",--(KeuzeZakelijk="ja"),IF(E21="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H21" s="20" t="n">
+      <c r="H21" s="22" t="n">
         <f aca="false">IF(G21="ja",F21*C21,0)</f>
         <v>0</v>
       </c>
-      <c r="I21" s="38"/>
+      <c r="I21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="49"/>
-      <c r="C22" s="50"/>
+      <c r="B22" s="55"/>
+      <c r="C22" s="56"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
-      <c r="F22" s="48" t="n">
+      <c r="F22" s="54" t="n">
         <f aca="false">IF(D22="Sectie I",$G$12,IF(D22="Sectie II",$G$13,IF(D22="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
         <v>0</v>
       </c>
-      <c r="G22" s="51" t="str">
+      <c r="G22" s="57" t="str">
         <f aca="false">IF(B22="","",IF(IF(E22="Altijd",1,IF(E22="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E22="Zakelijk",--(KeuzeZakelijk="ja"),IF(E22="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H22" s="20" t="n">
+      <c r="H22" s="22" t="n">
         <f aca="false">IF(G22="ja",F22*C22,0)</f>
         <v>0</v>
       </c>
-      <c r="I22" s="38"/>
+      <c r="I22" s="34"/>
     </row>
     <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="4"/>
@@ -2667,10 +3040,10 @@
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="43" t="s">
-        <v>72</v>
-      </c>
-      <c r="H23" s="22" t="n">
+      <c r="G23" s="49" t="s">
+        <v>92</v>
+      </c>
+      <c r="H23" s="25" t="n">
         <f aca="false">SUM(H17:H22)</f>
         <v>0</v>
       </c>
@@ -2688,7 +3061,7 @@
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="13" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
@@ -2699,154 +3072,154 @@
       <c r="I25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="D26" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="E26" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F26" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G26" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="H26" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="I26" s="23" t="s">
-        <v>52</v>
+      <c r="B26" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="F26" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="G26" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="H26" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="I26" s="26" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="49" t="s">
-        <v>77</v>
-      </c>
-      <c r="C27" s="18" t="n">
+      <c r="B27" s="55" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="19" t="n">
         <v>750</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="F27" s="52" t="n">
+        <v>99</v>
+      </c>
+      <c r="F27" s="58" t="n">
         <f aca="false">IF(D27="woning",AantalWoningen,IF(D27="project",1,0))</f>
         <v>1</v>
       </c>
-      <c r="G27" s="51" t="str">
+      <c r="G27" s="57" t="str">
         <f aca="false">IF(B27="","",IF(IF(E27="Altijd",1,IF(E27="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E27="Zakelijk",--(KeuzeZakelijk="ja"),IF(E27="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v>ja</v>
       </c>
-      <c r="H27" s="20" t="n">
+      <c r="H27" s="22" t="n">
         <f aca="false">IF(G27="ja",F27*C27,0)</f>
         <v>750</v>
       </c>
-      <c r="I27" s="38" t="s">
-        <v>80</v>
+      <c r="I27" s="34" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="49"/>
-      <c r="C28" s="18"/>
+      <c r="B28" s="55"/>
+      <c r="C28" s="19"/>
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
-      <c r="F28" s="52" t="n">
+      <c r="F28" s="58" t="n">
         <f aca="false">IF(D28="woning",AantalWoningen,IF(D28="project",1,0))</f>
         <v>0</v>
       </c>
-      <c r="G28" s="51" t="str">
+      <c r="G28" s="57" t="str">
         <f aca="false">IF(B28="","",IF(IF(E28="Altijd",1,IF(E28="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E28="Zakelijk",--(KeuzeZakelijk="ja"),IF(E28="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H28" s="20" t="n">
+      <c r="H28" s="22" t="n">
         <f aca="false">IF(G28="ja",F28*C28,0)</f>
         <v>0</v>
       </c>
-      <c r="I28" s="38"/>
+      <c r="I28" s="34"/>
     </row>
     <row r="29" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="49"/>
-      <c r="C29" s="18"/>
+      <c r="B29" s="55"/>
+      <c r="C29" s="19"/>
       <c r="D29" s="15"/>
       <c r="E29" s="15"/>
-      <c r="F29" s="52" t="n">
+      <c r="F29" s="58" t="n">
         <f aca="false">IF(D29="woning",AantalWoningen,IF(D29="project",1,0))</f>
         <v>0</v>
       </c>
-      <c r="G29" s="51" t="str">
+      <c r="G29" s="57" t="str">
         <f aca="false">IF(B29="","",IF(IF(E29="Altijd",1,IF(E29="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E29="Zakelijk",--(KeuzeZakelijk="ja"),IF(E29="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H29" s="20" t="n">
+      <c r="H29" s="22" t="n">
         <f aca="false">IF(G29="ja",F29*C29,0)</f>
         <v>0</v>
       </c>
-      <c r="I29" s="38"/>
+      <c r="I29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="49"/>
-      <c r="C30" s="18"/>
+      <c r="B30" s="55"/>
+      <c r="C30" s="19"/>
       <c r="D30" s="15"/>
       <c r="E30" s="15"/>
-      <c r="F30" s="52" t="n">
+      <c r="F30" s="58" t="n">
         <f aca="false">IF(D30="woning",AantalWoningen,IF(D30="project",1,0))</f>
         <v>0</v>
       </c>
-      <c r="G30" s="51" t="str">
+      <c r="G30" s="57" t="str">
         <f aca="false">IF(B30="","",IF(IF(E30="Altijd",1,IF(E30="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E30="Zakelijk",--(KeuzeZakelijk="ja"),IF(E30="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H30" s="20" t="n">
+      <c r="H30" s="22" t="n">
         <f aca="false">IF(G30="ja",F30*C30,0)</f>
         <v>0</v>
       </c>
-      <c r="I30" s="38"/>
+      <c r="I30" s="34"/>
     </row>
     <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="49"/>
-      <c r="C31" s="18"/>
+      <c r="B31" s="55"/>
+      <c r="C31" s="19"/>
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
-      <c r="F31" s="52" t="n">
+      <c r="F31" s="58" t="n">
         <f aca="false">IF(D31="woning",AantalWoningen,IF(D31="project",1,0))</f>
         <v>0</v>
       </c>
-      <c r="G31" s="51" t="str">
+      <c r="G31" s="57" t="str">
         <f aca="false">IF(B31="","",IF(IF(E31="Altijd",1,IF(E31="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E31="Zakelijk",--(KeuzeZakelijk="ja"),IF(E31="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H31" s="20" t="n">
+      <c r="H31" s="22" t="n">
         <f aca="false">IF(G31="ja",F31*C31,0)</f>
         <v>0</v>
       </c>
-      <c r="I31" s="38"/>
+      <c r="I31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="49"/>
-      <c r="C32" s="18"/>
+      <c r="B32" s="55"/>
+      <c r="C32" s="19"/>
       <c r="D32" s="15"/>
       <c r="E32" s="15"/>
-      <c r="F32" s="52" t="n">
+      <c r="F32" s="58" t="n">
         <f aca="false">IF(D32="woning",AantalWoningen,IF(D32="project",1,0))</f>
         <v>0</v>
       </c>
-      <c r="G32" s="51" t="str">
+      <c r="G32" s="57" t="str">
         <f aca="false">IF(B32="","",IF(IF(E32="Altijd",1,IF(E32="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E32="Zakelijk",--(KeuzeZakelijk="ja"),IF(E32="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
         <v/>
       </c>
-      <c r="H32" s="20" t="n">
+      <c r="H32" s="22" t="n">
         <f aca="false">IF(G32="ja",F32*C32,0)</f>
         <v>0</v>
       </c>
-      <c r="I32" s="38"/>
+      <c r="I32" s="34"/>
     </row>
     <row r="33" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="4"/>
@@ -2854,10 +3227,10 @@
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="43" t="s">
-        <v>72</v>
-      </c>
-      <c r="H33" s="22" t="n">
+      <c r="G33" s="49" t="s">
+        <v>92</v>
+      </c>
+      <c r="H33" s="25" t="n">
         <f aca="false">SUM(H27:H32)</f>
         <v>750</v>
       </c>
@@ -2874,29 +3247,49 @@
       <c r="I34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="31" t="s">
-        <v>81</v>
-      </c>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="32" t="n">
+      <c r="B35" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="36" t="n">
         <f aca="false">G12+G13+H23+H33</f>
         <v>1471.44072</v>
       </c>
-      <c r="I35" s="33"/>
+      <c r="I35" s="37"/>
     </row>
     <row r="36" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="4"/>
+      <c r="B36" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
+      <c r="H36" s="22" t="n">
+        <f aca="false">H35*C6</f>
+        <v>0</v>
+      </c>
       <c r="I36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="25" t="n">
+        <f aca="false">H35+H36</f>
+        <v>1471.44072</v>
+      </c>
+      <c r="I37" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2950,17 +3343,17 @@
     <tabColor rgb="FFC98A00"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:I36"/>
+  <dimension ref="B1:I45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2977,7 +3370,7 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2989,7 +3382,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -3011,46 +3404,52 @@
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
-      <c r="G5" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="44" t="str">
+      <c r="G5" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="50" t="str">
         <f aca="false">IF(I5="ja","OK","CONTROLEREN")</f>
-        <v>CONTROLEREN</v>
-      </c>
-      <c r="I5" s="16" t="s">
-        <v>12</v>
+        <v>OK</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="B6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>105</v>
+      </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="53" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
+    <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="59" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="59"/>
     </row>
     <row r="8" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="4"/>
@@ -3063,42 +3462,40 @@
       <c r="I8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="54" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="B9" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="60"/>
+      <c r="I9" s="60"/>
     </row>
     <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="G10" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="H10" s="26"/>
-      <c r="I10" s="23" t="s">
-        <v>52</v>
+      <c r="B10" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="26" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="45" t="s">
-        <v>53</v>
+      <c r="B11" s="51" t="s">
+        <v>111</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -3110,491 +3507,618 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" s="46" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="D12" s="47" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="48" t="n">
-        <f aca="false">AanneemsomIncl*D12</f>
-        <v>101640</v>
-      </c>
-      <c r="G12" s="20" t="n">
-        <f aca="false">F12*C12</f>
-        <v>508.2</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="C12" s="61" t="n">
+        <v>0.00227</v>
+      </c>
+      <c r="D12" s="61" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="E12" s="62" t="s">
+        <v>112</v>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
       <c r="H12" s="4"/>
-      <c r="I12" s="38" t="s">
-        <v>86</v>
+      <c r="I12" s="34" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="46" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="D13" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="48" t="n">
-        <f aca="false">AanneemsomIncl*D13</f>
-        <v>508200</v>
-      </c>
-      <c r="G13" s="20" t="n">
-        <f aca="false">F13*C13</f>
-        <v>203.28</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="C13" s="61" t="n">
+        <v>0.00321</v>
+      </c>
+      <c r="D13" s="61" t="n">
+        <v>0.00354</v>
+      </c>
+      <c r="E13" s="62" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
       <c r="H13" s="4"/>
-      <c r="I13" s="38" t="s">
-        <v>86</v>
+      <c r="I13" s="34" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
+      <c r="B14" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" s="61" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="D14" s="61" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="E14" s="62" t="s">
+        <v>115</v>
+      </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="54" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
+      <c r="I14" s="34"/>
+    </row>
+    <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="61" t="n">
+        <v>0.00321</v>
+      </c>
+      <c r="D15" s="61" t="n">
+        <v>0.00321</v>
+      </c>
+      <c r="E15" s="62" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="34" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C16" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="G16" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="H16" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>52</v>
-      </c>
+      <c r="B16" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="61" t="n">
+        <v>0.00568</v>
+      </c>
+      <c r="D16" s="61" t="n">
+        <v>0.00757</v>
+      </c>
+      <c r="E16" s="62" t="s">
+        <v>121</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="34"/>
     </row>
     <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="49" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="50" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="F17" s="48" t="n">
-        <f aca="false">IF(D17="Sectie I",$G$12,IF(D17="Sectie II",$G$13,IF(D17="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
-        <v>203.28</v>
-      </c>
-      <c r="G17" s="51" t="str">
-        <f aca="false">IF(B17="","",IF(IF(E17="Altijd",1,IF(E17="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E17="Zakelijk",--(KeuzeZakelijk="ja"),IF(E17="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
+      <c r="B17" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="C17" s="61" t="n">
+        <v>0.00343</v>
+      </c>
+      <c r="D17" s="61" t="n">
+        <v>0.00458</v>
+      </c>
+      <c r="E17" s="62" t="s">
+        <v>121</v>
+      </c>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="34"/>
+    </row>
+    <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" s="61" t="n">
+        <v>0.00903</v>
+      </c>
+      <c r="D18" s="61" t="n">
+        <v>0.00903</v>
+      </c>
+      <c r="E18" s="62" t="s">
+        <v>124</v>
+      </c>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="34" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19" s="61" t="n">
+        <v>0.00343</v>
+      </c>
+      <c r="D19" s="61" t="n">
+        <v>0.00343</v>
+      </c>
+      <c r="E19" s="62" t="s">
+        <v>121</v>
+      </c>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="34" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" s="60"/>
+      <c r="D21" s="60"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="60"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="60"/>
+      <c r="I21" s="60"/>
+    </row>
+    <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="63" t="str">
+        <f aca="false">WB_Regeling</f>
+        <v>Particulier nieuwbouw – verkoop met grond</v>
+      </c>
+      <c r="E22" s="63"/>
+      <c r="F22" s="63"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="4"/>
+      <c r="D23" s="63" t="str">
+        <f aca="false">WB_Hoog</f>
         <v>nee</v>
       </c>
-      <c r="H17" s="20" t="n">
-        <f aca="false">IF(G17="ja",F17*C17,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="38" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="49" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="50" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="48" t="n">
-        <f aca="false">IF(D18="Sectie I",$G$12,IF(D18="Sectie II",$G$13,IF(D18="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
-        <v>203.28</v>
-      </c>
-      <c r="G18" s="51" t="str">
-        <f aca="false">IF(B18="","",IF(IF(E18="Altijd",1,IF(E18="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E18="Zakelijk",--(KeuzeZakelijk="ja"),IF(E18="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v>nee</v>
-      </c>
-      <c r="H18" s="20" t="n">
-        <f aca="false">IF(G18="ja",F18*C18,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I18" s="38" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="C19" s="50" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="F19" s="48" t="n">
-        <f aca="false">IF(D19="Sectie I",$G$12,IF(D19="Sectie II",$G$13,IF(D19="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
-        <v>508.2</v>
-      </c>
-      <c r="G19" s="51" t="str">
-        <f aca="false">IF(B19="","",IF(IF(E19="Altijd",1,IF(E19="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E19="Zakelijk",--(KeuzeZakelijk="ja"),IF(E19="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v>nee</v>
-      </c>
-      <c r="H19" s="20" t="n">
-        <f aca="false">IF(G19="ja",F19*C19,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="38" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="49"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="48" t="n">
-        <f aca="false">IF(D20="Sectie I",$G$12,IF(D20="Sectie II",$G$13,IF(D20="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
-        <v>0</v>
-      </c>
-      <c r="G20" s="51" t="str">
-        <f aca="false">IF(B20="","",IF(IF(E20="Altijd",1,IF(E20="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E20="Zakelijk",--(KeuzeZakelijk="ja"),IF(E20="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H20" s="20" t="n">
-        <f aca="false">IF(G20="ja",F20*C20,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="38"/>
-    </row>
-    <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="49"/>
-      <c r="C21" s="50"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="48" t="n">
-        <f aca="false">IF(D21="Sectie I",$G$12,IF(D21="Sectie II",$G$13,IF(D21="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="51" t="str">
-        <f aca="false">IF(B21="","",IF(IF(E21="Altijd",1,IF(E21="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E21="Zakelijk",--(KeuzeZakelijk="ja"),IF(E21="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H21" s="20" t="n">
-        <f aca="false">IF(G21="ja",F21*C21,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I21" s="38"/>
-    </row>
-    <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="49"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="48" t="n">
-        <f aca="false">IF(D22="Sectie I",$G$12,IF(D22="Sectie II",$G$13,IF(D22="Aanneemsom incl. btw",AanneemsomIncl,0)))</f>
-        <v>0</v>
-      </c>
-      <c r="G22" s="51" t="str">
-        <f aca="false">IF(B22="","",IF(IF(E22="Altijd",1,IF(E22="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E22="Zakelijk",--(KeuzeZakelijk="ja"),IF(E22="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H22" s="20" t="n">
-        <f aca="false">IF(G22="ja",F22*C22,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I22" s="38"/>
-    </row>
-    <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="43" t="s">
-        <v>72</v>
-      </c>
-      <c r="H23" s="22" t="n">
-        <f aca="false">SUM(H17:H22)</f>
-        <v>0</v>
-      </c>
+      <c r="E23" s="63"/>
+      <c r="F23" s="63"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
       <c r="I23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="4"/>
+      <c r="B24" s="14" t="s">
+        <v>67</v>
+      </c>
       <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
+      <c r="D24" s="64" t="n">
+        <f aca="false">IFERROR(IF(WB_Hoog="ja",INDEX($D$12:$D$19,MATCH(WB_Regeling,$B$12:$B$19,0)),INDEX($C$12:$C$19,MATCH(WB_Regeling,$B$12:$B$19,0))),0)</f>
+        <v>0.00227</v>
+      </c>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="54" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="54"/>
-      <c r="D25" s="54"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="54"/>
+    <row r="25" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C25" s="4"/>
+      <c r="D25" s="63" t="str">
+        <f aca="false">IFERROR(INDEX($E$12:$E$19,MATCH(WB_Regeling,$B$12:$B$19,0)),"")</f>
+        <v>Koop- en aanneemsom incl. btw</v>
+      </c>
+      <c r="E25" s="63"/>
+      <c r="F25" s="63"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="D26" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="E26" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F26" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G26" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="H26" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="I26" s="23" t="s">
-        <v>52</v>
-      </c>
+      <c r="B26" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="65" t="n">
+        <f aca="false">IF(D25="Koop- en aanneemsom incl. btw",KoopAanneemIncl,IF(D25="Aanneemsom incl. btw",AanneemsomIncl,IF(D25="Koop- en aanneemsom excl. btw",AanneemsomExcl+GrondExcl,IF(D25="Aanneemsom excl. btw",AanneemsomExcl,0))))</f>
+        <v>605000</v>
+      </c>
+      <c r="E26" s="65"/>
+      <c r="F26" s="65"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="C27" s="18" t="n">
-        <v>700</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="F27" s="52" t="n">
-        <f aca="false">IF(D27="woning",AantalWoningen,IF(D27="project",1,0))</f>
-        <v>1</v>
-      </c>
-      <c r="G27" s="51" t="str">
-        <f aca="false">IF(B27="","",IF(IF(E27="Altijd",1,IF(E27="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E27="Zakelijk",--(KeuzeZakelijk="ja"),IF(E27="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v>ja</v>
-      </c>
-      <c r="H27" s="20" t="n">
-        <f aca="false">IF(G27="ja",F27*C27,0)</f>
-        <v>700</v>
-      </c>
-      <c r="I27" s="38" t="s">
-        <v>86</v>
-      </c>
+      <c r="B27" s="66" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="25" t="n">
+        <f aca="false">D26*D24</f>
+        <v>1373.35</v>
+      </c>
+      <c r="I27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="49"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="52" t="n">
-        <f aca="false">IF(D28="woning",AantalWoningen,IF(D28="project",1,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G28" s="51" t="str">
-        <f aca="false">IF(B28="","",IF(IF(E28="Altijd",1,IF(E28="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E28="Zakelijk",--(KeuzeZakelijk="ja"),IF(E28="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H28" s="20" t="n">
-        <f aca="false">IF(G28="ja",F28*C28,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I28" s="38"/>
-    </row>
-    <row r="29" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="49"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="52" t="n">
-        <f aca="false">IF(D29="woning",AantalWoningen,IF(D29="project",1,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G29" s="51" t="str">
-        <f aca="false">IF(B29="","",IF(IF(E29="Altijd",1,IF(E29="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E29="Zakelijk",--(KeuzeZakelijk="ja"),IF(E29="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H29" s="20" t="n">
-        <f aca="false">IF(G29="ja",F29*C29,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I29" s="38"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="60" t="s">
+        <v>132</v>
+      </c>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="60"/>
+      <c r="G29" s="60"/>
+      <c r="H29" s="60"/>
+      <c r="I29" s="60"/>
     </row>
     <row r="30" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="49"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="52" t="n">
-        <f aca="false">IF(D30="woning",AantalWoningen,IF(D30="project",1,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G30" s="51" t="str">
-        <f aca="false">IF(B30="","",IF(IF(E30="Altijd",1,IF(E30="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E30="Zakelijk",--(KeuzeZakelijk="ja"),IF(E30="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H30" s="20" t="n">
-        <f aca="false">IF(G30="ja",F30*C30,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I30" s="38"/>
+      <c r="B30" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E30" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="I30" s="26" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="49"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="52" t="n">
-        <f aca="false">IF(D31="woning",AantalWoningen,IF(D31="project",1,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G31" s="51" t="str">
-        <f aca="false">IF(B31="","",IF(IF(E31="Altijd",1,IF(E31="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E31="Zakelijk",--(KeuzeZakelijk="ja"),IF(E31="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H31" s="20" t="n">
-        <f aca="false">IF(G31="ja",F31*C31,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I31" s="38"/>
+      <c r="B31" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C31" s="19" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D31" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="22" t="n">
+        <f aca="false">C31*D31</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="34" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="49"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="52" t="n">
-        <f aca="false">IF(D32="woning",AantalWoningen,IF(D32="project",1,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G32" s="51" t="str">
-        <f aca="false">IF(B32="","",IF(IF(E32="Altijd",1,IF(E32="Hoogbouw",--(KeuzeHoogbouw="ja"),IF(E32="Zakelijk",--(KeuzeZakelijk="ja"),IF(E32="Bouwtijd &gt; 3 jaar",--(KeuzeBouwtijd="ja"),0))))=1,"ja","nee"))</f>
-        <v/>
-      </c>
-      <c r="H32" s="20" t="n">
-        <f aca="false">IF(G32="ja",F32*C32,0)</f>
-        <v>0</v>
-      </c>
-      <c r="I32" s="38"/>
+      <c r="B32" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="C32" s="19" t="n">
+        <v>911</v>
+      </c>
+      <c r="D32" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="22" t="n">
+        <f aca="false">C32*D32</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="34" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
+      <c r="B33" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C33" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D33" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="34" t="s">
+        <v>141</v>
+      </c>
       <c r="F33" s="4"/>
-      <c r="G33" s="43" t="s">
-        <v>72</v>
-      </c>
+      <c r="G33" s="4"/>
       <c r="H33" s="22" t="n">
-        <f aca="false">SUM(H27:H32)</f>
-        <v>700</v>
-      </c>
-      <c r="I33" s="4"/>
+        <f aca="false">C33*D33</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="34" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="B34" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>500</v>
+      </c>
+      <c r="D34" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="34" t="s">
+        <v>141</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-    </row>
-    <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="31" t="s">
-        <v>91</v>
-      </c>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="32" t="n">
-        <f aca="false">G12+G13+H23+H33</f>
-        <v>1411.48</v>
-      </c>
-      <c r="I35" s="33"/>
+      <c r="H34" s="22" t="n">
+        <f aca="false">C34*D34</f>
+        <v>0</v>
+      </c>
+      <c r="I34" s="34" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C35" s="19" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D35" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="22" t="n">
+        <f aca="false">C35*D35</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="34" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="B36" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="C36" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D36" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="34" t="s">
+        <v>141</v>
+      </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
+      <c r="H36" s="22" t="n">
+        <f aca="false">C36*D36</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="34" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C37" s="19" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D37" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="22" t="n">
+        <f aca="false">C37*D37</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="34" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C38" s="19" t="n">
+        <v>644</v>
+      </c>
+      <c r="D38" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="22" t="n">
+        <f aca="false">C38*D38</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="34" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C39" s="19" t="n">
+        <v>4018</v>
+      </c>
+      <c r="D39" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="22" t="n">
+        <f aca="false">C39*D39</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="34" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="49" t="s">
+        <v>92</v>
+      </c>
+      <c r="H40" s="25" t="n">
+        <f aca="false">SUM(H31:H39)</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="4"/>
+    </row>
+    <row r="41" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+    </row>
+    <row r="42" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+    </row>
+    <row r="43" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="35" t="s">
+        <v>153</v>
+      </c>
+      <c r="C43" s="37"/>
+      <c r="D43" s="37"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="37"/>
+      <c r="G43" s="37"/>
+      <c r="H43" s="36" t="n">
+        <f aca="false">H27+H40</f>
+        <v>1373.35</v>
+      </c>
+      <c r="I43" s="37"/>
+    </row>
+    <row r="44" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="22" t="n">
+        <f aca="false">H43*C6</f>
+        <v>288.4035</v>
+      </c>
+      <c r="I44" s="4"/>
+    </row>
+    <row r="45" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="25" t="n">
+        <f aca="false">H43+H44</f>
+        <v>1661.7535</v>
+      </c>
+      <c r="I45" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="13">
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="B7:I7"/>
     <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B15:I15"/>
-    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="B29:I29"/>
   </mergeCells>
   <conditionalFormatting sqref="H5">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
@@ -3604,21 +4128,18 @@
       <formula>H5&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <conditionalFormatting sqref="B12:E19">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>$B12=WB_Regeling</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5" type="list">
       <formula1>"ja,nee"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D17:D22" type="list">
-      <formula1>"Sectie I,Sectie II,Aanneemsom incl. btw"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E17:E22 E27:E32" type="list">
-      <formula1>"Altijd,Hoogbouw,Zakelijk,Bouwtijd &gt; 3 jaar,Nooit"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D27:D32" type="list">
-      <formula1>"woning,project"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E12:E19" type="list">
+      <formula1>"Koop- en aanneemsom incl. btw,Aanneemsom incl. btw,Koop- en aanneemsom excl. btw,Aanneemsom excl. btw"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -3627,7 +4148,7 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter>&amp;C&amp;"Arial,Regular"Heijmans Vastgoed | Tarieven Woningborg&amp;R&amp;"Arial,Regular"Pagina &amp;P van &amp;N</oddFooter>
+    <oddFooter>&amp;C&amp;"Arial,Regular"Heijmans Vastgoed | Tarieven Woningborg 2027&amp;R&amp;"Arial,Regular"Pagina &amp;P van &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -3637,12 +4158,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:C12"/>
+  <dimension ref="B1:C15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="120"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3653,74 +4174,96 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>92</v>
+        <v>155</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="55" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="56" t="s">
-        <v>94</v>
+      <c r="B5" s="68" t="s">
+        <v>156</v>
+      </c>
+      <c r="C5" s="69" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="55" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" s="56" t="s">
-        <v>96</v>
+      <c r="B6" s="68" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="69" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="55" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="56" t="s">
-        <v>98</v>
+      <c r="B7" s="68" t="s">
+        <v>160</v>
+      </c>
+      <c r="C7" s="69" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="55" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="56" t="s">
-        <v>100</v>
-      </c>
+      <c r="B8" s="68"/>
+      <c r="C8" s="70"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="55"/>
-      <c r="C9" s="56"/>
+      <c r="B9" s="68"/>
+      <c r="C9" s="68" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="55" t="s">
-        <v>101</v>
-      </c>
-      <c r="C10" s="56" t="s">
-        <v>102</v>
+      <c r="B10" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" s="69" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="55" t="s">
-        <v>103</v>
-      </c>
-      <c r="C11" s="56" t="s">
-        <v>104</v>
+      <c r="B11" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" s="69" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="55" t="s">
-        <v>101</v>
-      </c>
-      <c r="C12" s="56" t="s">
-        <v>105</v>
+      <c r="B12" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" s="69" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="C13" s="69" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="C14" s="69" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="C15" s="69" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>